<commit_message>
- Added Circuit Data to load parameters button
-  ui/ux improvements
</commit_message>
<xml_diff>
--- a/AE pyTools.extension/AE pyTools.Tab/Electrical.panel/Circuits1.stack/Circuit Tools.pulldown/Load Electrical Parameters.pushbutton/Content/ELEC SHARED PARAM TABLE.xlsx
+++ b/AE pyTools.extension/AE pyTools.Tab/Electrical.panel/Circuits1.stack/Circuit Tools.pulldown/Load Electrical Parameters.pushbutton/Content/ELEC SHARED PARAM TABLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aevelina\CED_Extensions\AE pyTools.extension\AE pyTools.Tab\Electrical.panel\Circuits1.stack\Circuit Tools.pulldown\Load Electrical Parameters.pushbutton\Content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917F13C7-3E2E-493C-891B-48AE8A52ADA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE4DF8C-E0F0-4EC8-ACC9-CBC5520A00B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32115" yWindow="5400" windowWidth="17355" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21855" yWindow="1710" windowWidth="29445" windowHeight="17685" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameter List" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="486">
   <si>
     <t>GUID</t>
   </si>
@@ -1499,6 +1499,12 @@
   </si>
   <si>
     <t>CKT_Length Makeup_CED</t>
+  </si>
+  <si>
+    <t>0e0811fc-86f1-4fd1-85f6-2a8ba53deb06</t>
+  </si>
+  <si>
+    <t>Circuit Data_CED</t>
   </si>
 </sst>
 </file>
@@ -1590,7 +1596,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1612,6 +1618,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1897,7 +1906,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultColWidth="66" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.5703125" style="2" customWidth="1"/>
@@ -2926,6 +2935,35 @@
         <v>35</v>
       </c>
     </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>484</v>
+      </c>
+      <c r="B36" s="1">
+        <v>35</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H38">
@@ -2933,22 +2971,22 @@
     </sortState>
   </autoFilter>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="F2:F35" xr:uid="{06D99139-2FA3-4AFB-B1C3-3BEE2A9AAD12}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="F2:F36" xr:uid="{06D99139-2FA3-4AFB-B1C3-3BEE2A9AAD12}">
       <formula1>ParamValues6</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="G2:G35" xr:uid="{1151C22F-EEEC-41FC-9B99-4E6AF0576CD2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="G2:G36" xr:uid="{1151C22F-EEEC-41FC-9B99-4E6AF0576CD2}">
       <formula1>ParamValues7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="H2:H35" xr:uid="{616A26CB-D9F9-4D1C-BA1B-E708E2CBE0E9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="H2:H36" xr:uid="{616A26CB-D9F9-4D1C-BA1B-E708E2CBE0E9}">
       <formula1>ParamValues8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="I2:I35" xr:uid="{B1E7E558-C3C7-40E8-8539-FFB9D8F8545E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="I2:I36" xr:uid="{B1E7E558-C3C7-40E8-8539-FFB9D8F8545E}">
       <formula1>ParamValues13</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="D2:D35" xr:uid="{827EEA15-0EC2-40C8-B587-AD980D20E9D0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="D2:D36" xr:uid="{827EEA15-0EC2-40C8-B587-AD980D20E9D0}">
       <formula1>ParamValues4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="E2:E35" xr:uid="{4E58A52C-D07C-4F2B-B4F2-F5CE0A750771}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="E2:E36" xr:uid="{4E58A52C-D07C-4F2B-B4F2-F5CE0A750771}">
       <formula1>INDIRECT(D2)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2960,6 +2998,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5390B230-261E-478F-825D-AC56AA77CC58}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -4832,6 +4871,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ce2a17a-c0eb-4821-a205-2297eefe49d7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010050F8A84B685D8A4A986E703CF63AF792" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2fa97ab612b8c94963ad725742f68d96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1ce2a17a-c0eb-4821-a205-2297eefe49d7" xmlns:ns3="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8fd2c164260f873fa57e921d57f91808" ns2:_="" ns3:_="">
     <xsd:import namespace="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
@@ -5038,27 +5097,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ce2a17a-c0eb-4821-a205-2297eefe49d7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADC3DD0-5BD5-40CE-B970-48D4CA313F4F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F0BD034-2603-47A7-897F-4421320EF50F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f"/>
+    <ds:schemaRef ds:uri="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0E6C32A-332A-47F8-AA61-6F8F7495A83A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5075,23 +5133,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F0BD034-2603-47A7-897F-4421320EF50F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f"/>
-    <ds:schemaRef ds:uri="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADC3DD0-5BD5-40CE-B970-48D4CA313F4F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UI framework/browser polish + MergeCircuits compatibility fix after develop merge (#35)
*Adds the new Circuit Manager UI surface (Circuit Browser + Alerts Browser) and supporting CEDElectrical application/infrastructure layers and shared UI resources.

* Refactors Wire Circuited Elements and Calculate Circuits to use the new operation flow, updates startup dockable-panel registration for Circuit Browser, 

* Applies ElementId compatibility hardening across existing tools (MergeCircuits, Sync One Line, Color Circuits by Panel). Includes related parameter/refdata updates and system-calculation behavior adjustments.
</commit_message>
<xml_diff>
--- a/AE pyTools.extension/AE pyTools.Tab/Electrical.panel/Circuits1.stack/Circuit Tools.pulldown/Load Electrical Parameters.pushbutton/Content/ELEC SHARED PARAM TABLE.xlsx
+++ b/AE pyTools.extension/AE pyTools.Tab/Electrical.panel/Circuits1.stack/Circuit Tools.pulldown/Load Electrical Parameters.pushbutton/Content/ELEC SHARED PARAM TABLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aevelina\CED_Extensions\AE pyTools.extension\AE pyTools.Tab\Electrical.panel\Circuits1.stack\Circuit Tools.pulldown\Load Electrical Parameters.pushbutton\Content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{917F13C7-3E2E-493C-891B-48AE8A52ADA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE4DF8C-E0F0-4EC8-ACC9-CBC5520A00B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32115" yWindow="5400" windowWidth="17355" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="21855" yWindow="1710" windowWidth="29445" windowHeight="17685" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameter List" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="486">
   <si>
     <t>GUID</t>
   </si>
@@ -1499,6 +1499,12 @@
   </si>
   <si>
     <t>CKT_Length Makeup_CED</t>
+  </si>
+  <si>
+    <t>0e0811fc-86f1-4fd1-85f6-2a8ba53deb06</t>
+  </si>
+  <si>
+    <t>Circuit Data_CED</t>
   </si>
 </sst>
 </file>
@@ -1590,7 +1596,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1612,6 +1618,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1897,7 +1906,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultColWidth="66" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.5703125" style="2" customWidth="1"/>
@@ -2926,6 +2935,35 @@
         <v>35</v>
       </c>
     </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>484</v>
+      </c>
+      <c r="B36" s="1">
+        <v>35</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H38">
@@ -2933,22 +2971,22 @@
     </sortState>
   </autoFilter>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="F2:F35" xr:uid="{06D99139-2FA3-4AFB-B1C3-3BEE2A9AAD12}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="F2:F36" xr:uid="{06D99139-2FA3-4AFB-B1C3-3BEE2A9AAD12}">
       <formula1>ParamValues6</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="G2:G35" xr:uid="{1151C22F-EEEC-41FC-9B99-4E6AF0576CD2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="G2:G36" xr:uid="{1151C22F-EEEC-41FC-9B99-4E6AF0576CD2}">
       <formula1>ParamValues7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="H2:H35" xr:uid="{616A26CB-D9F9-4D1C-BA1B-E708E2CBE0E9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="H2:H36" xr:uid="{616A26CB-D9F9-4D1C-BA1B-E708E2CBE0E9}">
       <formula1>ParamValues8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="I2:I35" xr:uid="{B1E7E558-C3C7-40E8-8539-FFB9D8F8545E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="I2:I36" xr:uid="{B1E7E558-C3C7-40E8-8539-FFB9D8F8545E}">
       <formula1>ParamValues13</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="D2:D35" xr:uid="{827EEA15-0EC2-40C8-B587-AD980D20E9D0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="D2:D36" xr:uid="{827EEA15-0EC2-40C8-B587-AD980D20E9D0}">
       <formula1>ParamValues4</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="E2:E35" xr:uid="{4E58A52C-D07C-4F2B-B4F2-F5CE0A750771}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="E2:E36" xr:uid="{4E58A52C-D07C-4F2B-B4F2-F5CE0A750771}">
       <formula1>INDIRECT(D2)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2960,6 +2998,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5390B230-261E-478F-825D-AC56AA77CC58}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -4832,6 +4871,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ce2a17a-c0eb-4821-a205-2297eefe49d7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010050F8A84B685D8A4A986E703CF63AF792" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2fa97ab612b8c94963ad725742f68d96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1ce2a17a-c0eb-4821-a205-2297eefe49d7" xmlns:ns3="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8fd2c164260f873fa57e921d57f91808" ns2:_="" ns3:_="">
     <xsd:import namespace="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
@@ -5038,27 +5097,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ce2a17a-c0eb-4821-a205-2297eefe49d7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADC3DD0-5BD5-40CE-B970-48D4CA313F4F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F0BD034-2603-47A7-897F-4421320EF50F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f"/>
+    <ds:schemaRef ds:uri="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0E6C32A-332A-47F8-AA61-6F8F7495A83A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5075,23 +5133,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F0BD034-2603-47A7-897F-4421320EF50F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f"/>
-    <ds:schemaRef ds:uri="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADC3DD0-5BD5-40CE-B970-48D4CA313F4F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>